<commit_message>
docs(scoping): specify composition architecture for weight engine
Each product line has unique physics (different materials, components,
seam allowances). Single template rejected -- composition pattern with
shared utilities (fabric calc, cube volume, cover weights, packaging)
plus per-product modules. Dura-Last downgraded to LOW-MEDIUM (12 paths,
poly fiber only). Updated D4, Workstream 5 notes (both phases), and
Excel workbook.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/American Bedding - CPQ Discussion/American_Bedding_CPQ_Estimate.xlsx
+++ b/American Bedding - CPQ Discussion/American_Bedding_CPQ_Estimate.xlsx
@@ -95,7 +95,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -109,11 +109,39 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -163,6 +191,8 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -893,15 +923,15 @@
           <t>PHASE 1 (V1): HUBSPOT-NATIVE CPQ</t>
         </is>
       </c>
-      <c r="B4" s="8" t="n"/>
-      <c r="C4" s="8" t="n"/>
-      <c r="D4" s="8" t="n"/>
-      <c r="E4" s="8" t="n"/>
-      <c r="F4" s="8" t="n"/>
-      <c r="G4" s="8" t="n"/>
-      <c r="H4" s="8" t="n"/>
-      <c r="I4" s="8" t="n"/>
-      <c r="J4" s="8" t="n"/>
+      <c r="B4" s="21" t="n"/>
+      <c r="C4" s="21" t="n"/>
+      <c r="D4" s="21" t="n"/>
+      <c r="E4" s="21" t="n"/>
+      <c r="F4" s="21" t="n"/>
+      <c r="G4" s="21" t="n"/>
+      <c r="H4" s="21" t="n"/>
+      <c r="I4" s="21" t="n"/>
+      <c r="J4" s="22" t="n"/>
       <c r="K4" s="8" t="n"/>
       <c r="L4" s="8" t="n"/>
       <c r="M4" s="8" t="n"/>
@@ -1141,7 +1171,7 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>HIGHEST-COMPLEXITY WORKSTREAM. Validated 2026-04-04: no VBA, no external refs, no circular formulas. Dorm (HIGH -- 9-level nesting, 180+ paths), Camp (MED -- 48+ paths), Dura-Last (MED -- 12+ paths), SoFlux OX/Vinyl (LOW -- ~80% reuse). Open: 'Special Case Check with Delbert' in Dorm Mattress.</t>
+          <t>HIGHEST-COMPLEXITY WORKSTREAM. Composition architecture: shared utilities (fabricCalc, cubeVolume, coverWeights, packagingCalc) + one module per product line. Each product has unique physics -- no single template. Dorm (HIGH -- 180+ paths, innerspring/foam/batting/cover), Camp (MED -- 48 paths, 4 foam series + fire barrier), Dura-Last (LOW-MED -- 12 paths, poly fiber only), SoFlux OX/Vinyl (LOW -- covers only, ~95% shared base). Validated 2026-04-04: no VBA, no external refs, no circular formulas. Open: 'Special Case Check with Delbert' in Dorm Mattress.</t>
         </is>
       </c>
       <c r="K9" s="9" t="n"/>
@@ -1448,15 +1478,15 @@
           <t>PHASE 2 (V2): RAILWAY PRODUCTION PLATFORM</t>
         </is>
       </c>
-      <c r="B17" s="13" t="n"/>
-      <c r="C17" s="13" t="n"/>
-      <c r="D17" s="13" t="n"/>
-      <c r="E17" s="13" t="n"/>
-      <c r="F17" s="13" t="n"/>
-      <c r="G17" s="13" t="n"/>
-      <c r="H17" s="13" t="n"/>
-      <c r="I17" s="13" t="n"/>
-      <c r="J17" s="13" t="n"/>
+      <c r="B17" s="21" t="n"/>
+      <c r="C17" s="21" t="n"/>
+      <c r="D17" s="21" t="n"/>
+      <c r="E17" s="21" t="n"/>
+      <c r="F17" s="21" t="n"/>
+      <c r="G17" s="21" t="n"/>
+      <c r="H17" s="21" t="n"/>
+      <c r="I17" s="21" t="n"/>
+      <c r="J17" s="22" t="n"/>
       <c r="K17" s="13" t="n"/>
       <c r="L17" s="13" t="n"/>
       <c r="M17" s="13" t="n"/>
@@ -1549,7 +1579,7 @@
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>Code already exists from Phase 1 -- migration is refactor + test coverage. Dorm Mattress needs ~20 representative test cases covering 80% of paths. SoFlux/Vinyl share ~80% code. Target: 100% coverage for critical paths.</t>
+          <t>Refactor 5 product modules + shared utilities into Railway API. Composition architecture: shared layer (fabricCalc, cubeVolume, coverWeights, packagingCalc) + per-product modules (dormMattress, campMattress, duraLast, sofluxCover, vinylCover). Each product built and tested independently -- no single template. Unit test coverage for all calculation paths. Dorm Mattress sampling strategy for 180+ paths. SoFlux/Vinyl share ~95% of a base cover module.</t>
         </is>
       </c>
       <c r="K19" s="9" t="n"/>

</xml_diff>

<commit_message>
feat(scoping): update build_estimate.py and proposal for composition architecture
Rebuilt build_estimate.py to match current two-phase hybrid architecture
with composition pattern weight engine. Updated proposal with modular
engine description and cell-by-cell validation constraint. Re-pushed to
Gamma: https://gamma.app/docs/t2wq974mrfi484u

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/American Bedding - CPQ Discussion/American_Bedding_CPQ_Estimate.xlsx
+++ b/American Bedding - CPQ Discussion/American_Bedding_CPQ_Estimate.xlsx
@@ -19,8 +19,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="7">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="$#,##0"/>
+  </numFmts>
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,29 +31,62 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Arial"/>
       <b val="1"/>
+      <color rgb="001F4E79"/>
       <sz val="14"/>
     </font>
     <font>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
     <font>
-      <b val="1"/>
+      <name val="Arial"/>
+      <sz val="10"/>
     </font>
     <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <b val="1"/>
       <sz val="12"/>
     </font>
     <font>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00008000"/>
+      <sz val="10"/>
     </font>
     <font>
+      <name val="Arial"/>
       <color rgb="00808080"/>
+      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -60,14 +95,26 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="004472C4"/>
-        <bgColor rgb="004472C4"/>
+        <fgColor rgb="001F4E79"/>
+        <bgColor rgb="001F4E79"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-        <bgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00F2F2F2"/>
+        <bgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DAEEF3"/>
+        <bgColor rgb="00DAEEF3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00548235"/>
+        <bgColor rgb="00548235"/>
       </patternFill>
     </fill>
     <fill>
@@ -78,14 +125,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
-        <bgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
-        <bgColor rgb="00E2EFDA"/>
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -94,8 +141,20 @@
         <bgColor rgb="00F4B084"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+        <bgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -109,90 +168,62 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin"/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="8" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -561,7 +592,7 @@
   <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
     <col width="55" customWidth="1" min="3" max="3"/>
   </cols>
@@ -608,17 +639,17 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Investment</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Phase 1 (V1): ~$30,000 | Phase 2 (V2): ~$11,500 | Total: ~$41,500</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>~$18,000-$22,000 (reduced scope)</t>
         </is>
@@ -642,17 +673,17 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Freight Automation</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Full -- Kuebix API with dynamic weight calculation. Multi-carrier LTL rate shopping automated. Phase 1 via HubSpot custom code, Phase 2 migrates to production API for unlimited execution time.</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>None or partial -- manual Kuebix entry continues, or NetSuite-side integration (TPI scope).</t>
         </is>
@@ -666,7 +697,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Dynamic engine replicates Excel formula logic for all 5 product lines. Handles custom sizes. Validated: no VBA, no macros, no external refs. Dorm Mattress is highest complexity (9-level nesting, 180+ paths).</t>
+          <t>Modular engine with composition architecture: shared utilities + per-product modules. Each product has unique physics (Dorm: innerspring/foam/batting, Camp: foam series + fire barrier, Dura-Last: poly fiber, SoFlux/Vinyl: covers only). Validated: no VBA, no macros, no external refs.</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -676,17 +707,17 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>NetSuite Integration</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Bi-directional: product catalog sync, quote-to-estimate creation, estimate-to-sales-order conversion, credit hold check.</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Enhanced one-way: quote visibility in HubSpot. No quote creation from HubSpot.</t>
         </is>
@@ -710,17 +741,17 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Risk Level</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>MEDIUM -- 3-system integration. Kuebix API fully reviewed. Excel calculators validated. HubSpot 20s timeout is Phase 1 limitation, eliminated in Phase 2.</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>LOW -- simpler scope but does not solve the core pain point (4-system juggling).</t>
         </is>
@@ -744,17 +775,17 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Payback Period</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>Phase 1: 6-8 months on labor savings alone</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>12-18 months (visibility value harder to quantify)</t>
         </is>
@@ -778,39 +809,41 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>Future Phase Readiness</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>Strong foundation for government RFP automation, customer configurator, and external storefront.</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>Minimal -- future phase would still need to move quoting to HubSpot.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>Recommendation</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>HubSpot CPQ with hybrid architecture is recommended. The core pain point is 4-system juggling that costs Caleb 10-60 minutes per quote across 65 quotes/week. The alternative (enhanced visibility) does not reduce that workload. The recommended approach eliminates system-jumping entirely, automates freight calculation, and builds the foundation for future phases. Two-phase delivery gets reps quoting in HubSpot fast (Phase 1) then hardens the platform for long-term reliability (Phase 2). The Kuebix API and Excel calculators have both been fully reviewed and validated.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="3">
+    <mergeCell ref="A1:C1"/>
     <mergeCell ref="A18:C18"/>
+    <mergeCell ref="A17:C17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -825,28 +858,28 @@
   <dimension ref="A1:M31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="65" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
     <col width="55" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Hourly Rate:</t>
         </is>
       </c>
-      <c r="B1" t="n">
+      <c r="B1" s="8" t="n">
         <v>150</v>
       </c>
     </row>
@@ -901,40 +934,40 @@
           <t>Notes / Assumptions</t>
         </is>
       </c>
-      <c r="K3" s="6" t="inlineStr">
+      <c r="K3" s="9" t="inlineStr">
         <is>
           <t>Actual Hours</t>
         </is>
       </c>
-      <c r="L3" s="6" t="inlineStr">
+      <c r="L3" s="9" t="inlineStr">
         <is>
           <t>Actual Cost</t>
         </is>
       </c>
-      <c r="M3" s="6" t="inlineStr">
+      <c r="M3" s="9" t="inlineStr">
         <is>
           <t>Variance</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>PHASE 1 (V1): HUBSPOT-NATIVE CPQ</t>
         </is>
       </c>
-      <c r="B4" s="21" t="n"/>
-      <c r="C4" s="21" t="n"/>
-      <c r="D4" s="21" t="n"/>
-      <c r="E4" s="21" t="n"/>
-      <c r="F4" s="21" t="n"/>
-      <c r="G4" s="21" t="n"/>
-      <c r="H4" s="21" t="n"/>
-      <c r="I4" s="21" t="n"/>
-      <c r="J4" s="22" t="n"/>
-      <c r="K4" s="8" t="n"/>
-      <c r="L4" s="8" t="n"/>
-      <c r="M4" s="8" t="n"/>
+      <c r="B4" s="11" t="n"/>
+      <c r="C4" s="11" t="n"/>
+      <c r="D4" s="11" t="n"/>
+      <c r="E4" s="11" t="n"/>
+      <c r="F4" s="11" t="n"/>
+      <c r="G4" s="11" t="n"/>
+      <c r="H4" s="11" t="n"/>
+      <c r="I4" s="11" t="n"/>
+      <c r="J4" s="11" t="n"/>
+      <c r="K4" s="11" t="n"/>
+      <c r="L4" s="11" t="n"/>
+      <c r="M4" s="11" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -961,15 +994,15 @@
         <f>$B$1</f>
         <v/>
       </c>
-      <c r="G5" s="3">
+      <c r="G5" s="12">
         <f>C5*$B$1</f>
         <v/>
       </c>
-      <c r="H5" s="3">
+      <c r="H5" s="12">
         <f>D5*$B$1</f>
         <v/>
       </c>
-      <c r="I5" s="3">
+      <c r="I5" s="12">
         <f>E5*$B$1</f>
         <v/>
       </c>
@@ -978,9 +1011,9 @@
           <t>Commerce Hub Professional confirmed. Standard CPQ config with custom properties for manufacturing context. Approval workflows for discount overrides.</t>
         </is>
       </c>
-      <c r="K5" s="9" t="n"/>
-      <c r="L5" s="9" t="n"/>
-      <c r="M5" s="9">
+      <c r="K5" s="13" t="n"/>
+      <c r="L5" s="13" t="n"/>
+      <c r="M5" s="13">
         <f>IF(K5="","",K5-E5)</f>
         <v/>
       </c>
@@ -1010,15 +1043,15 @@
         <f>$B$1</f>
         <v/>
       </c>
-      <c r="G6" s="3">
+      <c r="G6" s="12">
         <f>C6*$B$1</f>
         <v/>
       </c>
-      <c r="H6" s="3">
+      <c r="H6" s="12">
         <f>D6*$B$1</f>
         <v/>
       </c>
-      <c r="I6" s="3">
+      <c r="I6" s="12">
         <f>E6*$B$1</f>
         <v/>
       </c>
@@ -1027,9 +1060,9 @@
           <t>Flat catalog -- one product per SKU. SuiteQL batch queries (1-2 API calls). HubSpot custom code trigger replaces n8n scheduled sync. OAuth 2.0 M2M auth.</t>
         </is>
       </c>
-      <c r="K6" s="9" t="n"/>
-      <c r="L6" s="9" t="n"/>
-      <c r="M6" s="9">
+      <c r="K6" s="13" t="n"/>
+      <c r="L6" s="13" t="n"/>
+      <c r="M6" s="13">
         <f>IF(K6="","",K6-E6)</f>
         <v/>
       </c>
@@ -1059,15 +1092,15 @@
         <f>$B$1</f>
         <v/>
       </c>
-      <c r="G7" s="3">
+      <c r="G7" s="12">
         <f>C7*$B$1</f>
         <v/>
       </c>
-      <c r="H7" s="3">
+      <c r="H7" s="12">
         <f>D7*$B$1</f>
         <v/>
       </c>
-      <c r="I7" s="3">
+      <c r="I7" s="12">
         <f>E7*$B$1</f>
         <v/>
       </c>
@@ -1076,9 +1109,9 @@
           <t>Bi-directional: HubSpot quote -&gt; NetSuite estimate -&gt; sales order -&gt; work order. Credit hold reads AR data. 1.25x ERP adjacency premium (existing integration). HubSpot custom code handles orchestration.</t>
         </is>
       </c>
-      <c r="K7" s="9" t="n"/>
-      <c r="L7" s="9" t="n"/>
-      <c r="M7" s="9">
+      <c r="K7" s="13" t="n"/>
+      <c r="L7" s="13" t="n"/>
+      <c r="M7" s="13">
         <f>IF(K7="","",K7-E7)</f>
         <v/>
       </c>
@@ -1108,15 +1141,15 @@
         <f>$B$1</f>
         <v/>
       </c>
-      <c r="G8" s="3">
+      <c r="G8" s="12">
         <f>C8*$B$1</f>
         <v/>
       </c>
-      <c r="H8" s="3">
+      <c r="H8" s="12">
         <f>D8*$B$1</f>
         <v/>
       </c>
-      <c r="I8" s="3">
+      <c r="I8" s="12">
         <f>E8*$B$1</f>
         <v/>
       </c>
@@ -1125,9 +1158,9 @@
           <t>Kuebix API fully reviewed (OpenAPI 3.0.2). Basic Auth. quickRate returns multi-carrier quotes. Full street address required. Origin routing for multiple warehouses. persist=false prevents phantom shipments. 20s HubSpot timeout risk for multi-line quotes.</t>
         </is>
       </c>
-      <c r="K8" s="9" t="n"/>
-      <c r="L8" s="9" t="n"/>
-      <c r="M8" s="9">
+      <c r="K8" s="13" t="n"/>
+      <c r="L8" s="13" t="n"/>
+      <c r="M8" s="13">
         <f>IF(K8="","",K8-E8)</f>
         <v/>
       </c>
@@ -1140,7 +1173,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Replicate Excel formula logic in HubSpot custom code for all 5 product lines: Dorm Mattress, Camp Mattress, Dura-Last Poly-Fiber, SoFlux OX Covers, Vinyl Covers. Panel calcs, fabric weight by cover type, foam weight by density/thickness, innerspring weight by size, batting, insulator pad, packaging. Cube volume for LTL/TL determination.</t>
+          <t>Composition architecture: shared utilities (fabricCalc, cubeVolume, coverWeights, packagingCalc) + one module per product line. Dorm Mattress (innerspring + foam + batting + cover), Camp Mattress (foam core + fire barrier), Dura-Last (poly fiber), SoFlux OX/Vinyl (covers only). Each validated cell-by-cell against its Excel file. Cube volume for LTL/TL determination.</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
@@ -1157,26 +1190,26 @@
         <f>$B$1</f>
         <v/>
       </c>
-      <c r="G9" s="3">
+      <c r="G9" s="12">
         <f>C9*$B$1</f>
         <v/>
       </c>
-      <c r="H9" s="3">
+      <c r="H9" s="12">
         <f>D9*$B$1</f>
         <v/>
       </c>
-      <c r="I9" s="3">
+      <c r="I9" s="12">
         <f>E9*$B$1</f>
         <v/>
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>HIGHEST-COMPLEXITY WORKSTREAM. Composition architecture: shared utilities (fabricCalc, cubeVolume, coverWeights, packagingCalc) + one module per product line. Each product has unique physics -- no single template. Dorm (HIGH -- 180+ paths, innerspring/foam/batting/cover), Camp (MED -- 48 paths, 4 foam series + fire barrier), Dura-Last (LOW-MED -- 12 paths, poly fiber only), SoFlux OX/Vinyl (LOW -- covers only, ~95% shared base). Validated 2026-04-04: no VBA, no external refs, no circular formulas. Open: 'Special Case Check with Delbert' in Dorm Mattress.</t>
-        </is>
-      </c>
-      <c r="K9" s="9" t="n"/>
-      <c r="L9" s="9" t="n"/>
-      <c r="M9" s="9">
+          <t>HIGHEST-COMPLEXITY WORKSTREAM. Composition architecture -- no single template. Each product has unique physics, seam allowances, and construction constants that cannot be derived by analogy. Dorm (HIGH -- 180+ paths, 9-level nesting), Camp (MED -- 48 paths, foam series + fire barrier), Dura-Last (LOW-MED -- 12 paths, poly fiber), SoFlux OX/Vinyl (LOW -- ~95% shared base). Validated 2026-04-04: no VBA, no external refs, no circular formulas. Open: "Special Case Check with Delbert" in Dorm Mattress.</t>
+        </is>
+      </c>
+      <c r="K9" s="13" t="n"/>
+      <c r="L9" s="13" t="n"/>
+      <c r="M9" s="13">
         <f>IF(K9="","",K9-E9)</f>
         <v/>
       </c>
@@ -1206,15 +1239,15 @@
         <f>$B$1</f>
         <v/>
       </c>
-      <c r="G10" s="3">
+      <c r="G10" s="12">
         <f>C10*$B$1</f>
         <v/>
       </c>
-      <c r="H10" s="3">
+      <c r="H10" s="12">
         <f>D10*$B$1</f>
         <v/>
       </c>
-      <c r="I10" s="3">
+      <c r="I10" s="12">
         <f>E10*$B$1</f>
         <v/>
       </c>
@@ -1223,9 +1256,9 @@
           <t>Reference: 5 NetSuite PDF examples. Must match header/footer, line item format, terms. HubSpot Flow theme supports custom properties. @media print CSS for PDF.</t>
         </is>
       </c>
-      <c r="K10" s="9" t="n"/>
-      <c r="L10" s="9" t="n"/>
-      <c r="M10" s="9">
+      <c r="K10" s="13" t="n"/>
+      <c r="L10" s="13" t="n"/>
+      <c r="M10" s="13">
         <f>IF(K10="","",K10-E10)</f>
         <v/>
       </c>
@@ -1255,26 +1288,26 @@
         <f>$B$1</f>
         <v/>
       </c>
-      <c r="G11" s="3">
+      <c r="G11" s="12">
         <f>C11*$B$1</f>
         <v/>
       </c>
-      <c r="H11" s="3">
+      <c r="H11" s="12">
         <f>D11*$B$1</f>
         <v/>
       </c>
-      <c r="I11" s="3">
+      <c r="I11" s="12">
         <f>E11*$B$1</f>
         <v/>
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>Tax may need external service for multi-state. Discount approval thresholds TBD at kickoff. Credit hold is read from NetSuite -- flags but does not hard-block. Fits within HubSpot custom code 20s limit.</t>
-        </is>
-      </c>
-      <c r="K11" s="9" t="n"/>
-      <c r="L11" s="9" t="n"/>
-      <c r="M11" s="9">
+          <t>Tax may need external service for multi-state. Discount approval thresholds TBD at kickoff. Credit hold reads NetSuite -- flags but does not hard-block. Fits within HubSpot custom code 20s limit.</t>
+        </is>
+      </c>
+      <c r="K11" s="13" t="n"/>
+      <c r="L11" s="13" t="n"/>
+      <c r="M11" s="13">
         <f>IF(K11="","",K11-E11)</f>
         <v/>
       </c>
@@ -1304,15 +1337,15 @@
         <f>$B$1</f>
         <v/>
       </c>
-      <c r="G12" s="3">
+      <c r="G12" s="12">
         <f>C12*$B$1</f>
         <v/>
       </c>
-      <c r="H12" s="3">
+      <c r="H12" s="12">
         <f>D12*$B$1</f>
         <v/>
       </c>
-      <c r="I12" s="3">
+      <c r="I12" s="12">
         <f>E12*$B$1</f>
         <v/>
       </c>
@@ -1321,9 +1354,9 @@
           <t>2-3 sessions. Emphasis on time savings. Admin guide covers HubSpot custom code monitoring and product sync. Record for onboarding.</t>
         </is>
       </c>
-      <c r="K12" s="9" t="n"/>
-      <c r="L12" s="9" t="n"/>
-      <c r="M12" s="9">
+      <c r="K12" s="13" t="n"/>
+      <c r="L12" s="13" t="n"/>
+      <c r="M12" s="13">
         <f>IF(K12="","",K12-E12)</f>
         <v/>
       </c>
@@ -1336,7 +1369,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>E2E integration testing across all 3 systems. Quote accuracy vs. NetSuite examples. Weight calc vs. Excel baselines. Freight vs. manual Kuebix lookups. UAT with Caleb and Don. 2-week hypercare.</t>
+          <t>E2E integration testing across all 3 systems. Quote accuracy vs. NetSuite examples. Weight calc vs. Excel baselines (cell-by-cell per product -- no cross-product shortcuts). Freight vs. manual Kuebix lookups. UAT with Caleb and Don. 2-week hypercare.</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
@@ -1353,15 +1386,15 @@
         <f>$B$1</f>
         <v/>
       </c>
-      <c r="G13" s="3">
+      <c r="G13" s="12">
         <f>C13*$B$1</f>
         <v/>
       </c>
-      <c r="H13" s="3">
+      <c r="H13" s="12">
         <f>D13*$B$1</f>
         <v/>
       </c>
-      <c r="I13" s="3">
+      <c r="I13" s="12">
         <f>E13*$B$1</f>
         <v/>
       </c>
@@ -1370,9 +1403,9 @@
           <t>Test matrix: product sync accuracy, weight calc per product line, freight quote accuracy, template rendering, NetSuite estimate creation, SO conversion, credit hold. 2 UAT sessions. Dorm Mattress sampling strategy for 180+ paths.</t>
         </is>
       </c>
-      <c r="K13" s="9" t="n"/>
-      <c r="L13" s="9" t="n"/>
-      <c r="M13" s="9">
+      <c r="K13" s="13" t="n"/>
+      <c r="L13" s="13" t="n"/>
+      <c r="M13" s="13">
         <f>IF(K13="","",K13-E13)</f>
         <v/>
       </c>
@@ -1402,15 +1435,15 @@
         <f>$B$1</f>
         <v/>
       </c>
-      <c r="G14" s="3">
+      <c r="G14" s="12">
         <f>C14*$B$1</f>
         <v/>
       </c>
-      <c r="H14" s="3">
+      <c r="H14" s="12">
         <f>D14*$B$1</f>
         <v/>
       </c>
-      <c r="I14" s="3">
+      <c r="I14" s="12">
         <f>E14*$B$1</f>
         <v/>
       </c>
@@ -1419,77 +1452,77 @@
           <t>~10% of total. Weekly syncs with Sarah-Beth. Milestone reviews at weeks 4, 8, and go-live. All change requests documented.</t>
         </is>
       </c>
-      <c r="K14" s="9" t="n"/>
-      <c r="L14" s="9" t="n"/>
-      <c r="M14" s="9">
+      <c r="K14" s="13" t="n"/>
+      <c r="L14" s="13" t="n"/>
+      <c r="M14" s="13">
         <f>IF(K14="","",K14-E14)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>PHASE 1 SUBTOTAL</t>
         </is>
       </c>
-      <c r="B15" s="11" t="n"/>
-      <c r="C15" s="11">
+      <c r="B15" s="15" t="n"/>
+      <c r="C15" s="14">
         <f>SUM(C5:C14)</f>
         <v/>
       </c>
-      <c r="D15" s="11">
+      <c r="D15" s="14">
         <f>SUM(D5:D14)</f>
         <v/>
       </c>
-      <c r="E15" s="11">
+      <c r="E15" s="14">
         <f>SUM(E5:E14)</f>
         <v/>
       </c>
-      <c r="F15" s="11">
+      <c r="F15" s="14">
         <f>$B$1</f>
         <v/>
       </c>
-      <c r="G15" s="11">
+      <c r="G15" s="16">
         <f>SUM(G5:G14)</f>
         <v/>
       </c>
-      <c r="H15" s="11">
+      <c r="H15" s="16">
         <f>SUM(H5:H14)</f>
         <v/>
       </c>
-      <c r="I15" s="11">
+      <c r="I15" s="16">
         <f>SUM(I5:I14)</f>
         <v/>
       </c>
-      <c r="J15" s="11" t="n"/>
-      <c r="K15" s="11">
+      <c r="J15" s="15" t="n"/>
+      <c r="K15" s="15">
         <f>SUM(K5:K14)</f>
         <v/>
       </c>
-      <c r="L15" s="11">
+      <c r="L15" s="15">
         <f>SUM(L5:L14)</f>
         <v/>
       </c>
-      <c r="M15" s="11" t="n"/>
+      <c r="M15" s="15" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="inlineStr">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>PHASE 2 (V2): RAILWAY PRODUCTION PLATFORM</t>
         </is>
       </c>
-      <c r="B17" s="21" t="n"/>
-      <c r="C17" s="21" t="n"/>
-      <c r="D17" s="21" t="n"/>
-      <c r="E17" s="21" t="n"/>
-      <c r="F17" s="21" t="n"/>
-      <c r="G17" s="21" t="n"/>
-      <c r="H17" s="21" t="n"/>
-      <c r="I17" s="21" t="n"/>
-      <c r="J17" s="22" t="n"/>
-      <c r="K17" s="13" t="n"/>
-      <c r="L17" s="13" t="n"/>
-      <c r="M17" s="13" t="n"/>
+      <c r="B17" s="18" t="n"/>
+      <c r="C17" s="18" t="n"/>
+      <c r="D17" s="18" t="n"/>
+      <c r="E17" s="18" t="n"/>
+      <c r="F17" s="18" t="n"/>
+      <c r="G17" s="18" t="n"/>
+      <c r="H17" s="18" t="n"/>
+      <c r="I17" s="18" t="n"/>
+      <c r="J17" s="18" t="n"/>
+      <c r="K17" s="18" t="n"/>
+      <c r="L17" s="18" t="n"/>
+      <c r="M17" s="18" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -1516,26 +1549,26 @@
         <f>$B$1</f>
         <v/>
       </c>
-      <c r="G18" s="3">
+      <c r="G18" s="12">
         <f>C18*$B$1</f>
         <v/>
       </c>
-      <c r="H18" s="3">
+      <c r="H18" s="12">
         <f>D18*$B$1</f>
         <v/>
       </c>
-      <c r="I18" s="3">
+      <c r="I18" s="12">
         <f>E18*$B$1</f>
         <v/>
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>Railway provides managed hosting with auto-deploy from git. Node.js or Python runtime. Environment variables for secrets (API keys, OAuth tokens). Health check endpoint for uptime monitoring.</t>
-        </is>
-      </c>
-      <c r="K18" s="9" t="n"/>
-      <c r="L18" s="9" t="n"/>
-      <c r="M18" s="9">
+          <t>Railway provides managed hosting with auto-deploy from git. Node.js or Python runtime. Environment variables for secrets. Health check endpoint for uptime monitoring.</t>
+        </is>
+      </c>
+      <c r="K18" s="13" t="n"/>
+      <c r="L18" s="13" t="n"/>
+      <c r="M18" s="13">
         <f>IF(K18="","",K18-E18)</f>
         <v/>
       </c>
@@ -1548,7 +1581,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Migrate all 5 product-line calculators from HubSpot custom code to Railway API. Refactor into modular, testable JavaScript/Python modules. Add comprehensive unit test coverage for all calculation paths. Dorm Mattress sampling strategy for 180+ paths.</t>
+          <t>Refactor 5 product modules + shared utilities into Railway API. Composition architecture: shared layer (fabricCalc, cubeVolume, coverWeights, packagingCalc) + per-product modules (dormMattress, campMattress, duraLast, sofluxCover, vinylCover). Each product built and tested independently.</t>
         </is>
       </c>
       <c r="C19" s="3" t="n">
@@ -1565,26 +1598,26 @@
         <f>$B$1</f>
         <v/>
       </c>
-      <c r="G19" s="3">
+      <c r="G19" s="12">
         <f>C19*$B$1</f>
         <v/>
       </c>
-      <c r="H19" s="3">
+      <c r="H19" s="12">
         <f>D19*$B$1</f>
         <v/>
       </c>
-      <c r="I19" s="3">
+      <c r="I19" s="12">
         <f>E19*$B$1</f>
         <v/>
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>Refactor 5 product modules + shared utilities into Railway API. Composition architecture: shared layer (fabricCalc, cubeVolume, coverWeights, packagingCalc) + per-product modules (dormMattress, campMattress, duraLast, sofluxCover, vinylCover). Each product built and tested independently -- no single template. Unit test coverage for all calculation paths. Dorm Mattress sampling strategy for 180+ paths. SoFlux/Vinyl share ~95% of a base cover module.</t>
-        </is>
-      </c>
-      <c r="K19" s="9" t="n"/>
-      <c r="L19" s="9" t="n"/>
-      <c r="M19" s="9">
+          <t>Code exists from Phase 1 -- migration is refactor + test coverage. Each module validated cell-by-cell against its own Excel file -- no cross-product shortcuts. Dorm needs ~20 representative test cases for 180+ paths. SoFlux/Vinyl share ~95% code. Target: 100% coverage for critical paths.</t>
+        </is>
+      </c>
+      <c r="K19" s="13" t="n"/>
+      <c r="L19" s="13" t="n"/>
+      <c r="M19" s="13">
         <f>IF(K19="","",K19-E19)</f>
         <v/>
       </c>
@@ -1597,7 +1630,7 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Migrate Kuebix quickRate orchestration to Railway API. Multi-line, multi-carrier quote assembly without timeout risk. Retry logic for carrier API failures. Response caching for repeat origin/destination/weight combos.</t>
+          <t>Migrate Kuebix quickRate orchestration to Railway API. Multi-line, multi-carrier quote assembly without timeout risk. Retry logic for carrier API failures. Response caching for repeat shipping lanes.</t>
         </is>
       </c>
       <c r="C20" s="3" t="n">
@@ -1614,26 +1647,26 @@
         <f>$B$1</f>
         <v/>
       </c>
-      <c r="G20" s="3">
+      <c r="G20" s="12">
         <f>C20*$B$1</f>
         <v/>
       </c>
-      <c r="H20" s="3">
+      <c r="H20" s="12">
         <f>D20*$B$1</f>
         <v/>
       </c>
-      <c r="I20" s="3">
+      <c r="I20" s="12">
         <f>E20*$B$1</f>
         <v/>
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
-          <t>Eliminates HubSpot 20s timeout constraint. Retry logic handles intermittent Kuebix API failures gracefully. Cache reduces API calls for repeat shipping lanes.</t>
-        </is>
-      </c>
-      <c r="K20" s="9" t="n"/>
-      <c r="L20" s="9" t="n"/>
-      <c r="M20" s="9">
+          <t>Eliminates HubSpot 20s timeout constraint. Retry logic handles intermittent Kuebix API failures. Cache reduces API calls for repeat lanes.</t>
+        </is>
+      </c>
+      <c r="K20" s="13" t="n"/>
+      <c r="L20" s="13" t="n"/>
+      <c r="M20" s="13">
         <f>IF(K20="","",K20-E20)</f>
         <v/>
       </c>
@@ -1663,26 +1696,26 @@
         <f>$B$1</f>
         <v/>
       </c>
-      <c r="G21" s="3">
+      <c r="G21" s="12">
         <f>C21*$B$1</f>
         <v/>
       </c>
-      <c r="H21" s="3">
+      <c r="H21" s="12">
         <f>D21*$B$1</f>
         <v/>
       </c>
-      <c r="I21" s="3">
+      <c r="I21" s="12">
         <f>E21*$B$1</f>
         <v/>
       </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
-          <t>OAuth 2.0 M2M token refresh automated. SuiteQL catalog extraction runs on schedule (Railway cron). Estimate/SO creation with retry. Full audit logging.</t>
-        </is>
-      </c>
-      <c r="K21" s="9" t="n"/>
-      <c r="L21" s="9" t="n"/>
-      <c r="M21" s="9">
+          <t>OAuth 2.0 M2M token refresh automated. SuiteQL catalog extraction on schedule. Estimate/SO creation with retry. Full audit logging.</t>
+        </is>
+      </c>
+      <c r="K21" s="13" t="n"/>
+      <c r="L21" s="13" t="n"/>
+      <c r="M21" s="13">
         <f>IF(K21="","",K21-E21)</f>
         <v/>
       </c>
@@ -1712,26 +1745,26 @@
         <f>$B$1</f>
         <v/>
       </c>
-      <c r="G22" s="3">
+      <c r="G22" s="12">
         <f>C22*$B$1</f>
         <v/>
       </c>
-      <c r="H22" s="3">
+      <c r="H22" s="12">
         <f>D22*$B$1</f>
         <v/>
       </c>
-      <c r="I22" s="3">
+      <c r="I22" s="12">
         <f>E22*$B$1</f>
         <v/>
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
-          <t>Simple HTTP calls from HubSpot custom code to Railway API. Minimal logic in HubSpot -- just trigger + response handling. Reduces HubSpot custom code complexity significantly.</t>
-        </is>
-      </c>
-      <c r="K22" s="9" t="n"/>
-      <c r="L22" s="9" t="n"/>
-      <c r="M22" s="9">
+          <t>Simple HTTP calls from HubSpot custom code to Railway API. Minimal logic in HubSpot -- just trigger + response handling.</t>
+        </is>
+      </c>
+      <c r="K22" s="13" t="n"/>
+      <c r="L22" s="13" t="n"/>
+      <c r="M22" s="13">
         <f>IF(K22="","",K22-E22)</f>
         <v/>
       </c>
@@ -1761,15 +1794,15 @@
         <f>$B$1</f>
         <v/>
       </c>
-      <c r="G23" s="3">
+      <c r="G23" s="12">
         <f>C23*$B$1</f>
         <v/>
       </c>
-      <c r="H23" s="3">
+      <c r="H23" s="12">
         <f>D23*$B$1</f>
         <v/>
       </c>
-      <c r="I23" s="3">
+      <c r="I23" s="12">
         <f>E23*$B$1</f>
         <v/>
       </c>
@@ -1778,9 +1811,9 @@
           <t>Regression against Phase 1 baseline ensures zero behavior change. Load test confirms production volume capacity. Updated admin guide and architecture docs.</t>
         </is>
       </c>
-      <c r="K23" s="9" t="n"/>
-      <c r="L23" s="9" t="n"/>
-      <c r="M23" s="9">
+      <c r="K23" s="13" t="n"/>
+      <c r="L23" s="13" t="n"/>
+      <c r="M23" s="13">
         <f>IF(K23="","",K23-E23)</f>
         <v/>
       </c>
@@ -1810,15 +1843,15 @@
         <f>$B$1</f>
         <v/>
       </c>
-      <c r="G24" s="3">
+      <c r="G24" s="12">
         <f>C24*$B$1</f>
         <v/>
       </c>
-      <c r="H24" s="3">
+      <c r="H24" s="12">
         <f>D24*$B$1</f>
         <v/>
       </c>
-      <c r="I24" s="3">
+      <c r="I24" s="12">
         <f>E24*$B$1</f>
         <v/>
       </c>
@@ -1827,142 +1860,142 @@
           <t>Lighter PM load than Phase 1. ~10% of Phase 2 hours.</t>
         </is>
       </c>
-      <c r="K24" s="9" t="n"/>
-      <c r="L24" s="9" t="n"/>
-      <c r="M24" s="9">
+      <c r="K24" s="13" t="n"/>
+      <c r="L24" s="13" t="n"/>
+      <c r="M24" s="13">
         <f>IF(K24="","",K24-E24)</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="10" t="inlineStr">
+      <c r="A25" s="14" t="inlineStr">
         <is>
           <t>PHASE 2 SUBTOTAL</t>
         </is>
       </c>
-      <c r="B25" s="11" t="n"/>
-      <c r="C25" s="11">
+      <c r="B25" s="15" t="n"/>
+      <c r="C25" s="14">
         <f>SUM(C18:C24)</f>
         <v/>
       </c>
-      <c r="D25" s="11">
+      <c r="D25" s="14">
         <f>SUM(D18:D24)</f>
         <v/>
       </c>
-      <c r="E25" s="11">
+      <c r="E25" s="14">
         <f>SUM(E18:E24)</f>
         <v/>
       </c>
-      <c r="F25" s="11">
+      <c r="F25" s="14">
         <f>$B$1</f>
         <v/>
       </c>
-      <c r="G25" s="11">
+      <c r="G25" s="16">
         <f>SUM(G18:G24)</f>
         <v/>
       </c>
-      <c r="H25" s="11">
+      <c r="H25" s="16">
         <f>SUM(H18:H24)</f>
         <v/>
       </c>
-      <c r="I25" s="11">
+      <c r="I25" s="16">
         <f>SUM(I18:I24)</f>
         <v/>
       </c>
-      <c r="J25" s="11" t="n"/>
-      <c r="K25" s="11">
+      <c r="J25" s="15" t="n"/>
+      <c r="K25" s="15">
         <f>SUM(K18:K24)</f>
         <v/>
       </c>
-      <c r="L25" s="11">
+      <c r="L25" s="15">
         <f>SUM(L18:L24)</f>
         <v/>
       </c>
-      <c r="M25" s="11" t="n"/>
+      <c r="M25" s="15" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="14" t="inlineStr">
+      <c r="A27" s="19" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="B27" s="15" t="n"/>
-      <c r="C27" s="15">
+      <c r="B27" s="20" t="n"/>
+      <c r="C27" s="21">
         <f>C15+C25</f>
         <v/>
       </c>
-      <c r="D27" s="15">
+      <c r="D27" s="21">
         <f>D15+D25</f>
         <v/>
       </c>
-      <c r="E27" s="15">
+      <c r="E27" s="21">
         <f>E15+E25</f>
         <v/>
       </c>
-      <c r="F27" s="15">
+      <c r="F27" s="20">
         <f>$B$1</f>
         <v/>
       </c>
-      <c r="G27" s="15">
+      <c r="G27" s="22">
         <f>G15+G25</f>
         <v/>
       </c>
-      <c r="H27" s="15">
+      <c r="H27" s="22">
         <f>H15+H25</f>
         <v/>
       </c>
-      <c r="I27" s="15">
+      <c r="I27" s="22">
         <f>I15+I25</f>
         <v/>
       </c>
-      <c r="J27" s="15" t="n"/>
-      <c r="K27" s="15">
+      <c r="J27" s="20" t="n"/>
+      <c r="K27" s="20">
         <f>K15+K25</f>
         <v/>
       </c>
-      <c r="L27" s="15">
+      <c r="L27" s="20">
         <f>L15+L25</f>
         <v/>
       </c>
-      <c r="M27" s="15" t="n"/>
+      <c r="M27" s="20" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+      <c r="A29" s="5" t="inlineStr">
         <is>
           <t>PHASE 1 FIXED FEE:</t>
         </is>
       </c>
-      <c r="I29" t="n">
+      <c r="I29" s="23" t="n">
         <v>30000</v>
       </c>
-      <c r="J29" s="5" t="inlineStr">
+      <c r="J29" s="24" t="inlineStr">
         <is>
           <t>Fixed fee. Client sees this number only -- no hours breakdown in proposal.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+      <c r="A30" s="5" t="inlineStr">
         <is>
           <t>PHASE 2 FIXED FEE:</t>
         </is>
       </c>
-      <c r="I30" t="n">
+      <c r="I30" s="23" t="n">
         <v>11500</v>
       </c>
-      <c r="J30" s="5" t="inlineStr">
+      <c r="J30" s="24" t="inlineStr">
         <is>
           <t>Fixed fee. Separate SOW or Phase 2 addendum.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="16" t="inlineStr">
+      <c r="A31" s="25" t="inlineStr">
         <is>
           <t>COMBINED FIXED FEE:</t>
         </is>
       </c>
-      <c r="I31" s="16">
+      <c r="I31" s="26">
         <f>I29+I30</f>
         <v/>
       </c>
@@ -1985,14 +2018,14 @@
   <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="45" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2038,7 +2071,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="17" t="n">
+      <c r="A2" s="3" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -2046,12 +2079,12 @@
           <t>HubSpot custom code 20-second execution timeout for complex multi-line quotes</t>
         </is>
       </c>
-      <c r="C2" s="17" t="inlineStr">
+      <c r="C2" s="27" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="D2" s="17" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -2066,59 +2099,59 @@
           <t>Test with largest known quote configurations in Phase 1. Manual fallback for edge cases. Phase 2 eliminates this risk entirely by migrating to Railway API (no execution limits).</t>
         </is>
       </c>
-      <c r="G2" s="17" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Consultant</t>
         </is>
       </c>
-      <c r="H2" s="17" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>Open -- Phase 1 risk</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="17" t="n">
+      <c r="A3" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Excel weight calculator edge cases -- 'Special Case Check with Delbert' in Dorm Mattress</t>
-        </is>
-      </c>
-      <c r="C3" s="17" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Excel weight calculator edge cases -- "Special Case Check with Delbert" in Dorm Mattress</t>
+        </is>
+      </c>
+      <c r="C3" s="27" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="D3" s="17" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>Undocumented business logic in Dorm Mattress calculator. #VALUE! errors noted. Edge cases may produce incorrect weights for specific configurations.</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Clarify with Caleb/Delbert at kickoff. Build Dorm Mattress calculator first. Sampling strategy for 180+ paths (~20 representative test cases covering 80% of paths). Validate against known weights.</t>
-        </is>
-      </c>
-      <c r="G3" s="17" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Clarify with Caleb/Delbert at kickoff. Build Dorm Mattress calculator first. Sampling strategy for 180+ paths (~20 representative test cases). Validate against known weights.</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>Consultant + Caleb</t>
         </is>
       </c>
-      <c r="H3" s="17" t="inlineStr">
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="17" t="n">
+      <c r="A4" s="3" t="n">
         <v>3</v>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -2126,12 +2159,12 @@
           <t>NetSuite data quality -- SKU duplicates, stale pricing, missing attributes from Jan 2026 launch</t>
         </is>
       </c>
-      <c r="C4" s="17" t="inlineStr">
+      <c r="C4" s="28" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D4" s="17" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2146,59 +2179,59 @@
           <t>NetSuite item data audit during Week 1. Define cleanup scope before building sync. SuiteQL queries validate data quality before bulk import. Flag items missing required fields.</t>
         </is>
       </c>
-      <c r="G4" s="17" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Consultant + Sarah-Beth</t>
         </is>
       </c>
-      <c r="H4" s="17" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="17" t="n">
+      <c r="A5" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Scope creep via Vesco/Kaitlynn relationship -- government RFP work creeps into Phase 1</t>
         </is>
       </c>
-      <c r="C5" s="17" t="inlineStr">
+      <c r="C5" s="28" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D5" s="17" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Informal requests bypass SOW. Government-specific requirements consume hours budgeted for CPQ. Don Reynolds enthusiasm for future phases pulls scope.</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>SOW signed by Mike Taylor or Patrick (budget authority). Phase boundaries iron-clad in SOW. All change requests documented. Weekly hours tracking visible to client.</t>
         </is>
       </c>
-      <c r="G5" s="17" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>Kyle + Mike</t>
         </is>
       </c>
-      <c r="H5" s="17" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="17" t="n">
+      <c r="A6" s="3" t="n">
         <v>5</v>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -2206,12 +2239,12 @@
           <t>NetSuite still stabilizing (launched Jan 1, 2026) -- API schema changes, TPI updates</t>
         </is>
       </c>
-      <c r="C6" s="17" t="inlineStr">
+      <c r="C6" s="28" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D6" s="17" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -2226,59 +2259,59 @@
           <t>Build against documented REST API (not custom SuiteScript). Version-lock API endpoints. Establish communication channel with TPI for change notifications.</t>
         </is>
       </c>
-      <c r="G6" s="17" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>Consultant</t>
         </is>
       </c>
-      <c r="H6" s="17" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="17" t="n">
+      <c r="A7" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Multiple shipping origins -- wrong origin = wrong freight = wrong price</t>
         </is>
       </c>
-      <c r="C7" s="17" t="inlineStr">
+      <c r="C7" s="27" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="D7" s="17" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>Incorrect origin address sent to Kuebix. Freight quotes are wrong. Customer receives inaccurate pricing. Trust and margin impact.</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>Map all warehouse addresses at kickoff. Define explicit routing rules. Test each origin with known Kuebix quotes. Default origin fallback if routing is ambiguous.</t>
         </is>
       </c>
-      <c r="G7" s="17" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>Consultant + Mike</t>
         </is>
       </c>
-      <c r="H7" s="17" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="17" t="n">
+      <c r="A8" s="3" t="n">
         <v>7</v>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -2286,12 +2319,12 @@
           <t>HubSpot CPQ limitations -- no calculated fields, no product variants, no native tax engine</t>
         </is>
       </c>
-      <c r="C8" s="17" t="inlineStr">
+      <c r="C8" s="27" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="D8" s="17" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2306,59 +2339,59 @@
           <t>Pre-compute all calculated values in custom code before quote is published. Use custom properties and filtered views for product selection. Tax logic in Ops Hub custom code.</t>
         </is>
       </c>
-      <c r="G8" s="17" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>Consultant</t>
         </is>
       </c>
-      <c r="H8" s="17" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="17" t="n">
+      <c r="A9" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Kuebix API rate limits undocumented -- high quote volume could hit throttling</t>
         </is>
       </c>
-      <c r="C9" s="17" t="inlineStr">
+      <c r="C9" s="27" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="D9" s="17" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>65 quotes/week plus revisions could exceed undocumented rate limits. Freight quotes fail or are throttled.</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>Confirm rate limits with Kuebix support. Implement response caching for repeat shipping lanes (Phase 2). Graceful fallback to manual entry.</t>
         </is>
       </c>
-      <c r="G9" s="17" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>Consultant</t>
         </is>
       </c>
-      <c r="H9" s="17" t="inlineStr">
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="n">
+      <c r="A10" s="3" t="n">
         <v>9</v>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -2366,12 +2399,12 @@
           <t>Adoption risk -- sales reps switching from NetSuite quoting to HubSpot quoting</t>
         </is>
       </c>
-      <c r="C10" s="17" t="inlineStr">
+      <c r="C10" s="27" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="D10" s="17" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -2386,59 +2419,59 @@
           <t>Executive mandate from Mike. Show concrete time savings in training. 2-week parallel run. Monitor adoption metrics. Caleb is motivated (described the pain).</t>
         </is>
       </c>
-      <c r="G10" s="17" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>Mike + Consultant</t>
         </is>
       </c>
-      <c r="H10" s="17" t="inlineStr">
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="17" t="n">
+      <c r="A11" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>Freight class determination per product is unclear or inconsistent</t>
         </is>
       </c>
-      <c r="C11" s="17" t="inlineStr">
+      <c r="C11" s="27" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="D11" s="17" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>Wrong freight class to Kuebix. Shipping costs systematically over or under estimated. Margin impact across all quotes.</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr">
         <is>
           <t>Confirm freight class source at kickoff. Document per product line. Validate against known Kuebix quotes.</t>
         </is>
       </c>
-      <c r="G11" s="17" t="inlineStr">
+      <c r="G11" s="4" t="inlineStr">
         <is>
           <t>Consultant + Caleb</t>
         </is>
       </c>
-      <c r="H11" s="17" t="inlineStr">
+      <c r="H11" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="17" t="n">
+      <c r="A12" s="3" t="n">
         <v>11</v>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -2446,12 +2479,12 @@
           <t>Budget authority anchored on Billy $25K verbal benchmark -- two-phase total of ~$41.5K creates sticker shock</t>
         </is>
       </c>
-      <c r="C12" s="17" t="inlineStr">
+      <c r="C12" s="27" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="D12" s="17" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -2463,64 +2496,64 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Frame $25K as pre-discovery estimate. Phase 1 at ~$30K is closer to anchor than previous $34.5K. Two-phase reduces upfront commitment. Value-based ROI framing: Phase 1 pays back in 6-8 months. Phase 2 is a natural follow-on after reps see value.</t>
-        </is>
-      </c>
-      <c r="G12" s="17" t="inlineStr">
+          <t>Frame $25K as pre-discovery estimate. Phase 1 at ~$30K is closer to anchor than previous $34.5K. Two-phase reduces upfront commitment. Value-based ROI framing: Phase 1 pays back in 6-8 months.</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>Kyle + Billy</t>
         </is>
       </c>
-      <c r="H12" s="17" t="inlineStr">
+      <c r="H12" s="3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="inlineStr">
+      <c r="A14" s="29" t="inlineStr">
         <is>
           <t>RESOLVED</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="inlineStr">
+      <c r="A15" s="30" t="inlineStr">
         <is>
           <t>--</t>
         </is>
       </c>
-      <c r="B15" s="20" t="inlineStr">
+      <c r="B15" s="30" t="inlineStr">
         <is>
           <t>Excel weight calculator logic more complex than analyzed -- VBA macros, external references, or circular formulas</t>
         </is>
       </c>
-      <c r="C15" s="19" t="inlineStr">
+      <c r="C15" s="30" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D15" s="19" t="inlineStr">
+      <c r="D15" s="30" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="E15" s="20" t="inlineStr">
+      <c r="E15" s="30" t="inlineStr">
         <is>
           <t>Dynamic weight engine blows past 44 hrs. Fixed fee untenable. Workstream 5 unbounded.</t>
         </is>
       </c>
-      <c r="F15" s="20" t="inlineStr">
+      <c r="F15" s="30" t="inlineStr">
         <is>
           <t>RESOLVED 2026-04-04: All 5 Excel files received and validated. No VBA, no external refs, no circular formulas. Dorm Mattress confirmed as highest complexity (9-level nesting, 180+ paths) but within estimate range.</t>
         </is>
       </c>
-      <c r="G15" s="19" t="inlineStr">
+      <c r="G15" s="30" t="inlineStr">
         <is>
           <t>Kyle</t>
         </is>
       </c>
-      <c r="H15" s="19" t="inlineStr">
+      <c r="H15" s="30" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
@@ -2537,601 +2570,688 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B63"/>
+  <dimension ref="A1:C64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="95" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="16" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Scope Assumptions</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>HubSpot Sales Hub Professional + Commerce Hub Professional (existing)</t>
         </is>
       </c>
+      <c r="C2" s="6" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>Operations Hub Professional required (separate license ~$800/mo -- enables custom code actions)</t>
         </is>
       </c>
+      <c r="C3" s="6" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Up to 700 products in HubSpot product library (flat catalog, one record per SKU)</t>
         </is>
       </c>
+      <c r="C4" s="6" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>NetSuite REST API access with OAuth 2.0 M2M credentials provided by client</t>
         </is>
       </c>
+      <c r="C5" s="6" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Kuebix API credentials (username, API key, 15-character Client ID) provided by client</t>
         </is>
       </c>
+      <c r="C6" s="6" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Railway cloud platform for production API hosting (~$5-20/mo -- Phase 2)</t>
         </is>
       </c>
+      <c r="C7" s="6" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Multiple shipping origin addresses -- client provides complete warehouse list with routing rules at kickoff</t>
         </is>
       </c>
+      <c r="C8" s="6" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>Freight class stored as a property per product in NetSuite or as a static lookup per product line</t>
         </is>
       </c>
+      <c r="C9" s="6" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Up to 30 custom properties across deals, quotes, and line items (overages are change orders)</t>
         </is>
       </c>
+      <c r="C10" s="6" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" t="n">
+      <c r="A11" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Phase 1: 10-12 weeks | Phase 2: 4-6 weeks (18 weeks total)</t>
         </is>
       </c>
+      <c r="C11" s="6" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" t="n">
+      <c r="A12" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>All work conducted remotely</t>
         </is>
       </c>
+      <c r="C12" s="6" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" t="n">
+      <c r="A13" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>Rate: $150/hr (internal tracking -- client sees fixed fee only)</t>
         </is>
       </c>
+      <c r="C13" s="6" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" t="n">
+      <c r="A14" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Phase 1 fixed fee: ~$30,000 -- 5 payments of $6,300 ($6,000 + 5% tech/admin) every 15 days, Net-15</t>
         </is>
       </c>
+      <c r="C14" s="6" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" t="n">
+      <c r="A15" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>Phase 2 fixed fee: ~$11,500 -- 3 payments of ~$4,027 (~$3,835 + 5% tech/admin) every 15 days, Net-15</t>
         </is>
       </c>
+      <c r="C15" s="6" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" t="n">
+      <c r="A16" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Dynamic weight calculation covers 5 product lines (Dorm, Camp, Dura-Last, SoFlux OX, Vinyl)</t>
         </is>
       </c>
+      <c r="C16" s="6" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" t="n">
+      <c r="A17" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>Excel calculators validated: no VBA, no external refs, no circular formulas (confirmed 2026-04-04)</t>
         </is>
       </c>
+      <c r="C17" s="6" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" t="n">
+      <c r="A18" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Weight engine uses composition architecture: shared utilities + per-product modules (not a single template)</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>Quote template matches current NetSuite format (5 PDF examples as reference)</t>
         </is>
       </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>18</v>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="C19" s="6" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>SOW signed by Mike Taylor (VP) or Patrick (CFO) -- budget authority</t>
         </is>
       </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>19</v>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="C20" s="6" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>Production code delivered as version-controlled codebase (not n8n workflows)</t>
         </is>
       </c>
+      <c r="C21" s="6" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="16" t="inlineStr">
+      <c r="A22" s="6" t="n"/>
+      <c r="B22" s="6" t="n"/>
+      <c r="C22" s="6" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>Out of Scope</t>
         </is>
       </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="n">
+      <c r="B23" s="6" t="n"/>
+      <c r="C23" s="6" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>Government RFP automation, compliance tracking, bid management (future phase)</t>
         </is>
       </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
+      <c r="C24" s="6" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>Customer-facing product configurator / guided selling decision tree (future phase)</t>
         </is>
       </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
+      <c r="C25" s="6" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>External storefront build (Shopify or HubSpot Commerce -- future phase)</t>
         </is>
       </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
+      <c r="C26" s="6" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B26" s="5" t="inlineStr">
+      <c r="B27" s="6" t="inlineStr">
         <is>
           <t>VoIP / call capture system selection or integration</t>
         </is>
       </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
+      <c r="C27" s="6" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B27" s="5" t="inlineStr">
+      <c r="B28" s="6" t="inlineStr">
         <is>
           <t>AI lead enrichment from call transcripts</t>
         </is>
       </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
+      <c r="C28" s="6" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B28" s="5" t="inlineStr">
+      <c r="B29" s="6" t="inlineStr">
         <is>
           <t>NetSuite reimplementation, new module deployment, or SuiteScript development</t>
         </is>
       </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
+      <c r="C29" s="6" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B29" s="5" t="inlineStr">
+      <c r="B30" s="6" t="inlineStr">
         <is>
           <t>Ongoing Kuebix TMS administration or carrier management</t>
         </is>
       </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="n">
+      <c r="C30" s="6" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B30" s="5" t="inlineStr">
+      <c r="B31" s="6" t="inlineStr">
         <is>
           <t>HubSpot Marketing Hub configuration or marketing automation</t>
         </is>
       </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="n">
+      <c r="C31" s="6" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="B31" s="5" t="inlineStr">
+      <c r="B32" s="6" t="inlineStr">
         <is>
           <t>Custom self-service pricing portal</t>
         </is>
       </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="n">
+      <c r="C32" s="6" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B32" s="5" t="inlineStr">
+      <c r="B33" s="6" t="inlineStr">
         <is>
           <t>Ongoing managed services beyond 2-week hypercare per phase</t>
         </is>
       </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="n">
+      <c r="C33" s="6" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="B33" s="5" t="inlineStr">
+      <c r="B34" s="6" t="inlineStr">
         <is>
           <t>HubSpot or NetSuite license procurement or tier changes (recommendations only)</t>
         </is>
       </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="n">
+      <c r="C34" s="6" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B34" s="5" t="inlineStr">
+      <c r="B35" s="6" t="inlineStr">
         <is>
           <t>Data migration from external systems beyond NetSuite product catalog sync</t>
         </is>
       </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="n">
+      <c r="C35" s="6" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="B35" s="5" t="inlineStr">
+      <c r="B36" s="6" t="inlineStr">
         <is>
           <t>TPI (NetSuite partner) coordination or management -- Sayer works directly in NetSuite</t>
         </is>
       </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="n">
+      <c r="C36" s="6" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="B36" s="5" t="inlineStr">
+      <c r="B37" s="6" t="inlineStr">
         <is>
           <t>n8n as production runtime (may be used for prototyping only)</t>
         </is>
       </c>
+      <c r="C37" s="6" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="16" t="inlineStr">
+      <c r="A38" s="6" t="n"/>
+      <c r="B38" s="6" t="n"/>
+      <c r="C38" s="6" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
         <is>
           <t>Client Responsibilities</t>
         </is>
       </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="n">
+      <c r="B39" s="6" t="n"/>
+      <c r="C39" s="6" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B39" s="5" t="inlineStr">
+      <c r="B40" s="6" t="inlineStr">
         <is>
           <t>Provide Kuebix API credentials (username, API key, 15-character Client ID)</t>
         </is>
       </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="n">
+      <c r="C40" s="6" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B40" s="5" t="inlineStr">
+      <c r="B41" s="6" t="inlineStr">
         <is>
           <t>Provide NetSuite admin access or create OAuth 2.0 M2M integration record with API permissions</t>
         </is>
       </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="n">
+      <c r="C41" s="6" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B41" s="5" t="inlineStr">
+      <c r="B42" s="6" t="inlineStr">
         <is>
           <t>Excel shipping calculator files -- RECEIVED AND VALIDATED (2026-04-04)</t>
         </is>
       </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="n">
+      <c r="C42" s="6" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B42" s="5" t="inlineStr">
+      <c r="B43" s="6" t="inlineStr">
         <is>
           <t>Provide complete warehouse address list with product/region routing rules</t>
         </is>
       </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="n">
+      <c r="C43" s="6" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B43" s="5" t="inlineStr">
+      <c r="B44" s="6" t="inlineStr">
         <is>
           <t>Confirm freight class per product line (or provide lookup reference)</t>
         </is>
       </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="n">
+      <c r="C44" s="6" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B44" s="5" t="inlineStr">
+      <c r="B45" s="6" t="inlineStr">
         <is>
           <t>Designate primary point of contact (Sarah-Beth recommended)</t>
         </is>
       </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="n">
+      <c r="C45" s="6" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B45" s="5" t="inlineStr">
+      <c r="B46" s="6" t="inlineStr">
         <is>
           <t>Ensure Caleb and Don availability for 2+ UAT sessions during weeks 9-10</t>
         </is>
       </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="n">
+      <c r="C46" s="6" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B46" s="5" t="inlineStr">
+      <c r="B47" s="6" t="inlineStr">
         <is>
           <t>SOW signed by Mike Taylor or Patrick (CFO) -- budget authority</t>
         </is>
       </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="n">
+      <c r="C47" s="6" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="B47" s="5" t="inlineStr">
+      <c r="B48" s="6" t="inlineStr">
         <is>
           <t>Validate 5-10 sample quotes against current NetSuite output during UAT</t>
         </is>
       </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="n">
+      <c r="C48" s="6" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B48" s="5" t="inlineStr">
+      <c r="B49" s="6" t="inlineStr">
         <is>
           <t>Provide 5-10 recent quotes with known freight costs for validation testing</t>
         </is>
       </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="n">
+      <c r="C49" s="6" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="B49" s="5" t="inlineStr">
-        <is>
-          <t>Clarify 'Special Case Check with Delbert' for Dorm Mattress calculator</t>
-        </is>
-      </c>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>Clarify "Special Case Check with Delbert" for Dorm Mattress calculator</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="16" t="inlineStr">
+      <c r="A51" s="6" t="n"/>
+      <c r="B51" s="6" t="n"/>
+      <c r="C51" s="6" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
         <is>
           <t>Open Items (Confirm During Kickoff)</t>
         </is>
       </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="n">
+      <c r="B52" s="6" t="n"/>
+      <c r="C52" s="6" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B52" s="5" t="inlineStr">
+      <c r="B53" s="6" t="inlineStr">
         <is>
           <t>NetSuite item types in use (InventoryItem vs. AssemblyItem vs. NonInventoryItem)</t>
         </is>
       </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="n">
+      <c r="C53" s="6" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B53" s="5" t="inlineStr">
+      <c r="B54" s="6" t="inlineStr">
         <is>
           <t>NetSuite price level structure (single vs. multiple price levels per customer tier)</t>
         </is>
       </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="n">
+      <c r="C54" s="6" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B54" s="5" t="inlineStr">
+      <c r="B55" s="6" t="inlineStr">
         <is>
           <t>Exact number and full street addresses of all shipping warehouses</t>
         </is>
       </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="n">
+      <c r="C55" s="6" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B55" s="5" t="inlineStr">
+      <c r="B56" s="6" t="inlineStr">
         <is>
           <t>Routing rules: which products or regions ship from which warehouse</t>
         </is>
       </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="n">
+      <c r="C56" s="6" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B56" s="5" t="inlineStr">
+      <c r="B57" s="6" t="inlineStr">
         <is>
           <t>Discount approval thresholds -- is 10% always automatic? Do higher discounts need approval?</t>
         </is>
       </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="n">
+      <c r="C57" s="6" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B57" s="5" t="inlineStr">
+      <c r="B58" s="6" t="inlineStr">
         <is>
           <t>Credit hold workflow details -- what triggers a hold, who can override, block vs. flag?</t>
         </is>
       </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="n">
+      <c r="C58" s="6" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B58" s="5" t="inlineStr">
+      <c r="B59" s="6" t="inlineStr">
         <is>
           <t>Quote validity period (30 days per current NetSuite quotes -- confirm)</t>
         </is>
       </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="n">
+      <c r="C59" s="6" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B59" s="5" t="inlineStr">
-        <is>
-          <t>Dorm Mattress: 'Special Case Check with Delbert' -- undocumented business logic for edge cases</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="n">
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>Dorm Mattress: "Special Case Check with Delbert" -- undocumented business logic for edge cases</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="B60" s="5" t="inlineStr">
+      <c r="B61" s="6" t="inlineStr">
         <is>
           <t>Dimensional data future-proofing -- carriers may require L x W x H per item</t>
         </is>
       </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="n">
+      <c r="C61" s="6" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B61" s="5" t="inlineStr">
+      <c r="B62" s="6" t="inlineStr">
         <is>
           <t>Kuebix rate limits and acceptable API call volume (confirm with Kuebix support)</t>
         </is>
       </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="n">
+      <c r="C62" s="6" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="B62" s="5" t="inlineStr">
+      <c r="B63" s="6" t="inlineStr">
         <is>
           <t>Operations Hub Professional -- client decision on adding this tier (required for Phase 1)</t>
         </is>
       </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="n">
+      <c r="C63" s="6" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B63" s="5" t="inlineStr">
+      <c r="B64" s="6" t="inlineStr">
         <is>
           <t>Railway hosting -- confirm client or Sayer hosts the production API (Phase 2)</t>
         </is>
       </c>
+      <c r="C64" s="6" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>